<commit_message>
Automation of speckle paramters from geometries, push to google sheets for KPIs
</commit_message>
<xml_diff>
--- a/capsule_areas.xlsx
+++ b/capsule_areas.xlsx
@@ -438,8 +438,8 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -465,12 +465,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>PRG_PAR_DependenciesDistance</t>
+          <t>PRG_PAR_MeanDistToExit</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>PRG_PAR_IdealDependenciesDistance</t>
+          <t>PRG_PAR_IdealDistToExit</t>
         </is>
       </c>
     </row>
@@ -484,16 +484,16 @@
         <v>46083.69052</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>7373800</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>82.90747</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3">
@@ -503,19 +503,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>138251.07156</v>
+        <v>230418.4526</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>17512860.12962</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>211.58414</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4">
@@ -528,16 +528,16 @@
         <v>92167.38103999999</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>8664400</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>86.90747</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -550,16 +550,16 @@
         <v>397011.0276399991</v>
       </c>
       <c r="C5" t="n">
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>30310741.57825989</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>244.4077011022096</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6">
@@ -572,16 +572,16 @@
         <v>53766.57948000003</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>0.35</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>6981508.123249996</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>473.2202196913585</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
@@ -594,16 +594,16 @@
         <v>46083.69052</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>5530400</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>98.90747</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8">
@@ -616,16 +616,16 @@
         <v>59668.03606000001</v>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>7748160.199500005</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>94.22593113372091</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9">
@@ -638,10 +638,10 @@
         <v>23041.84526</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>2027800</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -660,16 +660,16 @@
         <v>115109.5048700001</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>14947468.21176</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>294.0411970632529</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
     </row>
     <row r="11">
@@ -682,16 +682,16 @@
         <v>23041.84526</v>
       </c>
       <c r="C11" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>2534800</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>104.90747</v>
       </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -701,13 +701,11 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>994224.6722099991</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>1086392.053249999</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>103631938.2423899</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -745,7 +743,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>994224.67221</v>
+        <v>1086392.05325</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +772,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>994224.6722099958</v>
+        <v>1086392.053249996</v>
       </c>
     </row>
     <row r="8">
@@ -803,7 +801,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>994224.6722099958</v>
+        <v>1086392.053249996</v>
       </c>
     </row>
     <row r="12">
@@ -842,7 +840,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>138251.07156</v>
+        <v>230418.4526</v>
       </c>
     </row>
     <row r="16">
@@ -951,7 +949,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>994224.6722099958</v>
+        <v>1086392.053249996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PRG_PAR_ResourceConsRatio added to columns
</commit_message>
<xml_diff>
--- a/capsule_areas.xlsx
+++ b/capsule_areas.xlsx
@@ -431,15 +431,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,15 +461,20 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>PRG_PAR_ResourceConsRatio</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>PRG_PAR_GeometryWeight</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>PRG_PAR_MeanDistToExit</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>PRG_PAR_IdealDistToExit</t>
         </is>
@@ -487,12 +493,15 @@
         <v>0.1</v>
       </c>
       <c r="D2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E2" t="n">
         <v>7373800</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>82.90747</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>75</v>
       </c>
     </row>
@@ -509,12 +518,15 @@
         <v>0.4</v>
       </c>
       <c r="D3" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E3" t="n">
         <v>17512860.12962</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>211.58414</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>200</v>
       </c>
     </row>
@@ -531,12 +543,15 @@
         <v>0.15</v>
       </c>
       <c r="D4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E4" t="n">
         <v>8664400</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>86.90747</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>50</v>
       </c>
     </row>
@@ -553,12 +568,15 @@
         <v>0.16</v>
       </c>
       <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
         <v>30310741.57825989</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>244.4077011022096</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>250</v>
       </c>
     </row>
@@ -575,12 +593,15 @@
         <v>0.35</v>
       </c>
       <c r="D6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E6" t="n">
         <v>6981508.123249996</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>473.2202196913585</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>500</v>
       </c>
     </row>
@@ -597,12 +618,15 @@
         <v>0.3</v>
       </c>
       <c r="D7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E7" t="n">
         <v>5530400</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>98.90747</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>50</v>
       </c>
     </row>
@@ -619,12 +643,15 @@
         <v>0.5</v>
       </c>
       <c r="D8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E8" t="n">
         <v>7748160.199500005</v>
       </c>
-      <c r="E8" t="n">
+      <c r="F8" t="n">
         <v>94.22593113372091</v>
       </c>
-      <c r="F8" t="n">
+      <c r="G8" t="n">
         <v>100</v>
       </c>
     </row>
@@ -641,14 +668,17 @@
         <v>0.8</v>
       </c>
       <c r="D9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="E9" t="n">
         <v>2027800</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
       </c>
+      <c r="G9" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -663,12 +693,15 @@
         <v>0.25</v>
       </c>
       <c r="D10" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E10" t="n">
         <v>14947468.21176</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>294.0411970632529</v>
       </c>
-      <c r="F10" t="n">
+      <c r="G10" t="n">
         <v>300</v>
       </c>
     </row>
@@ -685,12 +718,15 @@
         <v>0.6</v>
       </c>
       <c r="D11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E11" t="n">
         <v>2534800</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>104.90747</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>100</v>
       </c>
     </row>
@@ -704,11 +740,12 @@
         <v>1086392.053249999</v>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="n">
         <v>103631938.2423899</v>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>